<commit_message>
fix: Improve server startup sequence and bot thread reliability
</commit_message>
<xml_diff>
--- a/לקוחות_רועי.xlsx
+++ b/לקוחות_רועי.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -972,6 +972,258 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>03/04/2026 22:12</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>נכנס לראשונה</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>03/04/2026 22:12</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>רמת גן</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>03/04/2026 22:31</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>נכנס לראשונה</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>03/04/2026 22:31</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>רמת גן</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>השכרה</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>03/04/2026 23:12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>נכנס לראשונה</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>03/04/2026 23:12</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>רמת גן</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>השכרה</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix bot and add dockerfile
</commit_message>
<xml_diff>
--- a/לקוחות_רועי.xlsx
+++ b/לקוחות_רועי.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1224,6 +1224,86 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04/04/2026 11:24</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>נכנס לראשונה</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04/04/2026 11:25</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Eliyo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>רמת גן</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>השכרה</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>חדש</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>לא ידוע</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>